<commit_message>
Want to add the make system
</commit_message>
<xml_diff>
--- a/Assets/GameAsset/Configs/Recipe.xlsx
+++ b/Assets/GameAsset/Configs/Recipe.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PROJECT\Unity\PackageExample\Assets\GameAsset\Configs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{40D150BD-908F-4502-BAF4-B644CE9FAFD8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB2B07C2-9A81-4D9E-86F7-281B1EA5C2CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="12710" yWindow="0" windowWidth="12980" windowHeight="15370" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -408,30 +408,30 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">

</xml_diff>